<commit_message>
Rimuove file obsoleti/di supporto non più necessari
</commit_message>
<xml_diff>
--- a/docs/Prodotti_Tracciato.xlsx
+++ b/docs/Prodotti_Tracciato.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E4839ADA-6F71-4EF7-A12F-32E593AC9677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B89FC5C1-EB60-4006-9A53-7E94E6108F6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12,7 +12,7 @@
     <sheet name="Guida" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Prodotti!$A$1:$R$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Prodotti!$A$1:$R$57</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
@@ -281,7 +281,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="173">
   <si>
     <t>sku_interno</t>
   </si>
@@ -337,49 +337,13 @@
     <t>note_interne</t>
   </si>
   <si>
-    <t>Acido Cloridrico 37%</t>
-  </si>
-  <si>
-    <t>HCl 37% - Tanica 25L</t>
-  </si>
-  <si>
-    <t>Tanica HDPE 25 litri</t>
-  </si>
-  <si>
     <t>semplice</t>
   </si>
   <si>
-    <t>Acidi</t>
-  </si>
-  <si>
     <t>kg</t>
   </si>
   <si>
-    <t>tanica</t>
-  </si>
-  <si>
-    <t>25.00</t>
-  </si>
-  <si>
-    <t>25.000</t>
-  </si>
-  <si>
-    <t>26.200</t>
-  </si>
-  <si>
-    <t>8012345678901</t>
-  </si>
-  <si>
-    <t>WOO-HCL-25L</t>
-  </si>
-  <si>
-    <t>45.00</t>
-  </si>
-  <si>
     <t>1</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Campo</t>
@@ -845,7 +809,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -861,13 +825,6 @@
       <family val="2"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF555555"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFCC0000"/>
@@ -875,7 +832,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -885,11 +842,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF2E4057"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEAF2FB"/>
       </patternFill>
     </fill>
   </fills>
@@ -905,14 +857,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1253,8 +1204,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:R58"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1327,655 +1277,643 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="I2" s="2" t="s">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2">
         <v>25</v>
       </c>
-      <c r="J2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
+      <c r="J2">
+        <v>25</v>
+      </c>
+      <c r="K2">
+        <v>25</v>
+      </c>
+      <c r="N2" s="4">
+        <v>51.3</v>
+      </c>
+      <c r="O2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G3" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I3">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="J3">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="K3">
-        <v>25</v>
-      </c>
-      <c r="N3" s="5">
-        <v>51.3</v>
+        <v>10</v>
+      </c>
+      <c r="N3" s="4">
+        <v>22.5</v>
       </c>
       <c r="O3" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P3" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="D4" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G4" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K4">
-        <v>10</v>
-      </c>
-      <c r="N4" s="5">
-        <v>22.5</v>
+        <v>5</v>
+      </c>
+      <c r="N4" s="4">
+        <v>11.88</v>
       </c>
       <c r="O4" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P4" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q4" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="D5" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F5" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G5" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H5" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>5</v>
-      </c>
-      <c r="N5" s="5">
-        <v>11.88</v>
+        <v>1</v>
+      </c>
+      <c r="N5" s="4">
+        <v>7.3770490000000004</v>
       </c>
       <c r="O5" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P5" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q5" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="D6" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F6" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G6" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="N6" s="5">
-        <v>7.3770490000000004</v>
+        <v>10</v>
+      </c>
+      <c r="N6" s="4">
+        <v>52.459015999999998</v>
       </c>
       <c r="O6" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P6" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G7" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H7" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I7">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J7">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K7">
-        <v>10</v>
-      </c>
-      <c r="N7" s="5">
-        <v>52.459015999999998</v>
+        <v>5</v>
+      </c>
+      <c r="N7" s="4">
+        <v>29.508196999999999</v>
       </c>
       <c r="O7" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P7" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q7" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="D8" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G8" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H8" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I8">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J8">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K8">
-        <v>5</v>
-      </c>
-      <c r="N8" s="5">
-        <v>29.508196999999999</v>
+        <v>10</v>
+      </c>
+      <c r="N8" s="4">
+        <v>43.442622999999998</v>
       </c>
       <c r="O8" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P8" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D9" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="E9" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F9" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G9" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H9" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K9">
-        <v>10</v>
-      </c>
-      <c r="N9" s="5">
-        <v>43.442622999999998</v>
+        <v>5</v>
+      </c>
+      <c r="N9" s="4">
+        <v>23.770491</v>
       </c>
       <c r="O9" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P9" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q9" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="D10" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F10" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G10" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H10" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K10">
-        <v>5</v>
-      </c>
-      <c r="N10" s="5">
-        <v>23.770491</v>
+        <v>1</v>
+      </c>
+      <c r="N10" s="4">
+        <v>9.0163930000000008</v>
       </c>
       <c r="O10" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P10" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q10" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="D11" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="E11" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F11" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="G11" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H11" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="J11">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="K11">
-        <v>1</v>
-      </c>
-      <c r="N11" s="5">
-        <v>9.0163930000000008</v>
+        <v>15</v>
+      </c>
+      <c r="N11" s="4">
+        <v>34.426229999999997</v>
       </c>
       <c r="O11" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P11" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="D12" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
       <c r="E12" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F12" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="G12" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H12" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I12">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="J12">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="K12">
-        <v>15</v>
-      </c>
-      <c r="N12" s="5">
-        <v>34.426229999999997</v>
+        <v>5</v>
+      </c>
+      <c r="N12" s="4">
+        <v>14.754098000000001</v>
       </c>
       <c r="O12" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P12" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q12" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="B13" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="D13" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="E13" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F13" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="G13" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H13" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K13">
-        <v>5</v>
-      </c>
-      <c r="N13" s="5">
-        <v>14.754098000000001</v>
+        <v>1</v>
+      </c>
+      <c r="N13" s="4">
+        <v>8.1967210000000001</v>
       </c>
       <c r="O13" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P13" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q13" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="D14" t="s">
-        <v>175</v>
+        <v>159</v>
       </c>
       <c r="E14" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F14" t="s">
+        <v>154</v>
+      </c>
+      <c r="G14" t="s">
+        <v>152</v>
+      </c>
+      <c r="H14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14">
+        <v>25</v>
+      </c>
+      <c r="J14">
+        <v>25</v>
+      </c>
+      <c r="K14">
+        <v>25</v>
+      </c>
+      <c r="N14" s="4">
+        <v>22.131148</v>
+      </c>
+      <c r="O14" t="s">
+        <v>20</v>
+      </c>
+      <c r="P14" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D15" t="s">
+        <v>167</v>
+      </c>
+      <c r="E15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" t="s">
+        <v>154</v>
+      </c>
+      <c r="G15" t="s">
+        <v>152</v>
+      </c>
+      <c r="H15" t="s">
+        <v>19</v>
+      </c>
+      <c r="I15">
+        <v>10</v>
+      </c>
+      <c r="J15">
+        <v>10</v>
+      </c>
+      <c r="K15">
+        <v>10</v>
+      </c>
+      <c r="N15" s="4">
+        <v>12.295082000000001</v>
+      </c>
+      <c r="O15" t="s">
+        <v>20</v>
+      </c>
+      <c r="P15" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" t="s">
+        <v>168</v>
+      </c>
+      <c r="D16" t="s">
         <v>166</v>
       </c>
-      <c r="G14" t="s">
-        <v>164</v>
-      </c>
-      <c r="H14" t="s">
-        <v>23</v>
-      </c>
-      <c r="I14">
-        <v>1</v>
-      </c>
-      <c r="J14">
-        <v>1</v>
-      </c>
-      <c r="K14">
-        <v>1</v>
-      </c>
-      <c r="N14" s="5">
-        <v>8.1967210000000001</v>
-      </c>
-      <c r="O14" t="s">
-        <v>31</v>
-      </c>
-      <c r="P14" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>65</v>
-      </c>
-      <c r="B15" t="s">
-        <v>121</v>
-      </c>
-      <c r="D15" t="s">
-        <v>171</v>
-      </c>
-      <c r="E15" t="s">
-        <v>21</v>
-      </c>
-      <c r="F15" t="s">
-        <v>166</v>
-      </c>
-      <c r="G15" t="s">
-        <v>164</v>
-      </c>
-      <c r="H15" t="s">
-        <v>23</v>
-      </c>
-      <c r="I15">
-        <v>25</v>
-      </c>
-      <c r="J15">
-        <v>25</v>
-      </c>
-      <c r="K15">
-        <v>25</v>
-      </c>
-      <c r="N15" s="5">
-        <v>22.131148</v>
-      </c>
-      <c r="O15" t="s">
-        <v>31</v>
-      </c>
-      <c r="P15" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>66</v>
-      </c>
-      <c r="B16" t="s">
-        <v>122</v>
-      </c>
-      <c r="D16" t="s">
-        <v>179</v>
-      </c>
       <c r="E16" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F16" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="G16" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H16" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I16">
         <v>10</v>
@@ -1986,172 +1924,172 @@
       <c r="K16">
         <v>10</v>
       </c>
-      <c r="N16" s="5">
-        <v>12.295082000000001</v>
+      <c r="N16" s="4">
+        <v>21.311475000000002</v>
       </c>
       <c r="O16" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P16" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="B17" t="s">
-        <v>180</v>
+        <v>111</v>
       </c>
       <c r="D17" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="E17" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F17" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="G17" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H17" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I17">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J17">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K17">
-        <v>10</v>
-      </c>
-      <c r="N17" s="5">
-        <v>21.311475000000002</v>
+        <v>5</v>
+      </c>
+      <c r="N17" s="4">
+        <v>15.57</v>
       </c>
       <c r="O17" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P17" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q17" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B18" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="D18" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="E18" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F18" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="G18" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H18" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I18">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J18">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K18">
-        <v>5</v>
-      </c>
-      <c r="N18" s="5">
-        <v>15.57</v>
+        <v>1</v>
+      </c>
+      <c r="N18" s="4">
+        <v>6.5573769999999998</v>
       </c>
       <c r="O18" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P18" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q18" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="B19" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="D19" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="E19" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F19" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="G19" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H19" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J19">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K19">
-        <v>1</v>
-      </c>
-      <c r="N19" s="5">
-        <v>6.5573769999999998</v>
+        <v>5</v>
+      </c>
+      <c r="N19" s="4">
+        <v>85.245902000000001</v>
       </c>
       <c r="O19" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P19" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q19" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B20" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="D20" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="E20" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F20" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="G20" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H20" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I20">
         <v>5</v>
@@ -2162,700 +2100,700 @@
       <c r="K20">
         <v>5</v>
       </c>
-      <c r="N20" s="5">
-        <v>85.245902000000001</v>
+      <c r="N20" s="4">
+        <v>31.147541</v>
       </c>
       <c r="O20" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P20" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q20" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="B21" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="D21" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="E21" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F21" t="s">
+        <v>155</v>
+      </c>
+      <c r="G21" t="s">
+        <v>152</v>
+      </c>
+      <c r="H21" t="s">
+        <v>19</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+      <c r="J21">
+        <v>1</v>
+      </c>
+      <c r="K21">
+        <v>1</v>
+      </c>
+      <c r="N21" s="4">
+        <v>9.0163930000000008</v>
+      </c>
+      <c r="O21" t="s">
+        <v>20</v>
+      </c>
+      <c r="P21" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" t="s">
+        <v>116</v>
+      </c>
+      <c r="D22" t="s">
         <v>167</v>
       </c>
-      <c r="G21" t="s">
-        <v>164</v>
-      </c>
-      <c r="H21" t="s">
-        <v>23</v>
-      </c>
-      <c r="I21">
-        <v>5</v>
-      </c>
-      <c r="J21">
-        <v>5</v>
-      </c>
-      <c r="K21">
-        <v>5</v>
-      </c>
-      <c r="N21" s="5">
-        <v>31.147541</v>
-      </c>
-      <c r="O21" t="s">
-        <v>31</v>
-      </c>
-      <c r="P21" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>72</v>
-      </c>
-      <c r="B22" t="s">
-        <v>127</v>
-      </c>
-      <c r="D22" t="s">
-        <v>174</v>
-      </c>
       <c r="E22" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F22" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="G22" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H22" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J22">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K22">
-        <v>1</v>
-      </c>
-      <c r="N22" s="5">
-        <v>9.0163930000000008</v>
+        <v>10</v>
+      </c>
+      <c r="N22" s="4">
+        <v>18.032786999999999</v>
       </c>
       <c r="O22" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P22" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q22" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="B23" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="D23" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E23" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F23" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="G23" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H23" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I23">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J23">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K23">
-        <v>10</v>
-      </c>
-      <c r="N23" s="5">
-        <v>18.032786999999999</v>
+        <v>5</v>
+      </c>
+      <c r="N23" s="4">
+        <v>12.295082000000001</v>
       </c>
       <c r="O23" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P23" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q23" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="B24" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="D24" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="E24" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F24" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="G24" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H24" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I24">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J24">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K24">
-        <v>5</v>
-      </c>
-      <c r="N24" s="5">
-        <v>12.295082000000001</v>
+        <v>1</v>
+      </c>
+      <c r="N24" s="4">
+        <v>6.5573769999999998</v>
       </c>
       <c r="O24" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P24" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q24" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="B25" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="D25" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="E25" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F25" t="s">
+        <v>155</v>
+      </c>
+      <c r="G25" t="s">
+        <v>152</v>
+      </c>
+      <c r="H25" t="s">
+        <v>19</v>
+      </c>
+      <c r="I25">
+        <v>10</v>
+      </c>
+      <c r="J25">
+        <v>10</v>
+      </c>
+      <c r="K25">
+        <v>10</v>
+      </c>
+      <c r="N25" s="4">
+        <v>20.491803000000001</v>
+      </c>
+      <c r="O25" t="s">
+        <v>20</v>
+      </c>
+      <c r="P25" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>65</v>
+      </c>
+      <c r="B26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D26" t="s">
+        <v>159</v>
+      </c>
+      <c r="E26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" t="s">
+        <v>156</v>
+      </c>
+      <c r="G26" t="s">
+        <v>152</v>
+      </c>
+      <c r="H26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I26">
+        <v>25</v>
+      </c>
+      <c r="J26">
+        <v>25</v>
+      </c>
+      <c r="K26">
+        <v>25</v>
+      </c>
+      <c r="N26" s="4">
+        <v>40.163933999999998</v>
+      </c>
+      <c r="O26" t="s">
+        <v>20</v>
+      </c>
+      <c r="P26" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>66</v>
+      </c>
+      <c r="B27" t="s">
+        <v>121</v>
+      </c>
+      <c r="D27" t="s">
         <v>167</v>
       </c>
-      <c r="G25" t="s">
-        <v>164</v>
-      </c>
-      <c r="H25" t="s">
-        <v>23</v>
-      </c>
-      <c r="I25">
-        <v>1</v>
-      </c>
-      <c r="J25">
-        <v>1</v>
-      </c>
-      <c r="K25">
-        <v>1</v>
-      </c>
-      <c r="N25" s="5">
-        <v>6.5573769999999998</v>
-      </c>
-      <c r="O25" t="s">
-        <v>31</v>
-      </c>
-      <c r="P25" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q25" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>76</v>
-      </c>
-      <c r="B26" t="s">
-        <v>131</v>
-      </c>
-      <c r="D26" t="s">
-        <v>178</v>
-      </c>
-      <c r="E26" t="s">
-        <v>21</v>
-      </c>
-      <c r="F26" t="s">
-        <v>167</v>
-      </c>
-      <c r="G26" t="s">
-        <v>164</v>
-      </c>
-      <c r="H26" t="s">
-        <v>23</v>
-      </c>
-      <c r="I26">
-        <v>10</v>
-      </c>
-      <c r="J26">
-        <v>10</v>
-      </c>
-      <c r="K26">
-        <v>10</v>
-      </c>
-      <c r="N26" s="5">
-        <v>20.491803000000001</v>
-      </c>
-      <c r="O26" t="s">
-        <v>31</v>
-      </c>
-      <c r="P26" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q26" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>77</v>
-      </c>
-      <c r="B27" t="s">
-        <v>132</v>
-      </c>
-      <c r="D27" t="s">
-        <v>171</v>
-      </c>
       <c r="E27" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F27" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="G27" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H27" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I27">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="J27">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="K27">
-        <v>25</v>
-      </c>
-      <c r="N27" s="5">
-        <v>40.163933999999998</v>
+        <v>10</v>
+      </c>
+      <c r="N27" s="4">
+        <v>23.770492000000001</v>
       </c>
       <c r="O27" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P27" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q27" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B28" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="D28" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E28" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F28" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="G28" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H28" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I28">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J28">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K28">
-        <v>10</v>
-      </c>
-      <c r="N28" s="5">
-        <v>23.770492000000001</v>
+        <v>5</v>
+      </c>
+      <c r="N28" s="4">
+        <v>13.934426</v>
       </c>
       <c r="O28" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P28" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q28" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="B29" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="D29" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="E29" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F29" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="G29" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H29" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I29">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J29">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K29">
-        <v>5</v>
-      </c>
-      <c r="N29" s="5">
-        <v>13.934426</v>
+        <v>1</v>
+      </c>
+      <c r="N29" s="4">
+        <v>6.5573769999999998</v>
       </c>
       <c r="O29" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P29" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q29" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="B30" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="D30" t="s">
-        <v>183</v>
+        <v>170</v>
       </c>
       <c r="E30" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F30" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="G30" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H30" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I30">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J30">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K30">
-        <v>1</v>
-      </c>
-      <c r="N30" s="5">
-        <v>6.5573769999999998</v>
+        <v>5</v>
+      </c>
+      <c r="N30" s="4">
+        <v>16.393442</v>
       </c>
       <c r="O30" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P30" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q30" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="B31" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="D31" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="E31" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F31" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="G31" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H31" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I31">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J31">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K31">
-        <v>5</v>
-      </c>
-      <c r="N31" s="5">
-        <v>16.393442</v>
+        <v>1</v>
+      </c>
+      <c r="N31" s="4">
+        <v>7.3770490000000004</v>
       </c>
       <c r="O31" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P31" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q31" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="B32" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="D32" t="s">
-        <v>183</v>
+        <v>170</v>
       </c>
       <c r="E32" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F32" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="G32" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H32" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I32">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J32">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K32">
-        <v>1</v>
-      </c>
-      <c r="N32" s="5">
-        <v>7.3770490000000004</v>
+        <v>5</v>
+      </c>
+      <c r="N32" s="4">
+        <v>14.754098000000001</v>
       </c>
       <c r="O32" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P32" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q32" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="B33" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="D33" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="E33" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F33" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G33" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H33" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I33">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J33">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K33">
-        <v>5</v>
-      </c>
-      <c r="N33" s="5">
-        <v>14.754098000000001</v>
+        <v>1</v>
+      </c>
+      <c r="N33" s="4">
+        <v>7.3770490000000004</v>
       </c>
       <c r="O33" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P33" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q33" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="B34" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="D34" t="s">
-        <v>183</v>
+        <v>167</v>
       </c>
       <c r="E34" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F34" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G34" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H34" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I34">
+        <v>10</v>
+      </c>
+      <c r="J34">
+        <v>10</v>
+      </c>
+      <c r="K34">
+        <v>10</v>
+      </c>
+      <c r="N34" s="4">
+        <v>11.47541</v>
+      </c>
+      <c r="O34" t="s">
+        <v>20</v>
+      </c>
+      <c r="P34" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>74</v>
+      </c>
+      <c r="B35" t="s">
+        <v>129</v>
+      </c>
+      <c r="D35" t="s">
+        <v>171</v>
+      </c>
+      <c r="E35" t="s">
+        <v>18</v>
+      </c>
+      <c r="F35" t="s">
+        <v>157</v>
+      </c>
+      <c r="G35" t="s">
+        <v>152</v>
+      </c>
+      <c r="H35" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35">
         <v>1</v>
       </c>
-      <c r="J34">
+      <c r="J35">
         <v>1</v>
       </c>
-      <c r="K34">
+      <c r="K35">
         <v>1</v>
       </c>
-      <c r="N34" s="5">
-        <v>7.3770490000000004</v>
-      </c>
-      <c r="O34" t="s">
-        <v>31</v>
-      </c>
-      <c r="P34" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q34" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="35" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>85</v>
-      </c>
-      <c r="B35" t="s">
-        <v>140</v>
-      </c>
-      <c r="D35" t="s">
-        <v>179</v>
-      </c>
-      <c r="E35" t="s">
-        <v>21</v>
-      </c>
-      <c r="F35" t="s">
-        <v>169</v>
-      </c>
-      <c r="G35" t="s">
-        <v>164</v>
-      </c>
-      <c r="H35" t="s">
-        <v>23</v>
-      </c>
-      <c r="I35">
-        <v>10</v>
-      </c>
-      <c r="J35">
-        <v>10</v>
-      </c>
-      <c r="K35">
-        <v>10</v>
-      </c>
-      <c r="N35" s="5">
-        <v>11.47541</v>
+      <c r="N35" s="4">
+        <v>4.0999999999999996</v>
       </c>
       <c r="O35" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P35" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q35" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="B36" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="D36" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="E36" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F36" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G36" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H36" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I36">
         <v>1</v>
@@ -2866,352 +2804,352 @@
       <c r="K36">
         <v>1</v>
       </c>
-      <c r="N36" s="5">
-        <v>4.0999999999999996</v>
+      <c r="N36" s="4">
+        <v>8.1967210000000001</v>
       </c>
       <c r="O36" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P36" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q36" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="B37" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="D37" t="s">
-        <v>183</v>
+        <v>170</v>
       </c>
       <c r="E37" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F37" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G37" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H37" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I37">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J37">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K37">
-        <v>1</v>
-      </c>
-      <c r="N37" s="5">
-        <v>8.1967210000000001</v>
+        <v>5</v>
+      </c>
+      <c r="N37" s="4">
+        <v>14.754098000000001</v>
       </c>
       <c r="O37" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P37" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q37" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="B38" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="D38" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="E38" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F38" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G38" t="s">
-        <v>164</v>
-      </c>
-      <c r="H38" t="s">
-        <v>23</v>
-      </c>
-      <c r="I38">
-        <v>5</v>
-      </c>
-      <c r="J38">
-        <v>5</v>
-      </c>
-      <c r="K38">
-        <v>5</v>
-      </c>
-      <c r="N38" s="5">
-        <v>14.754098000000001</v>
+        <v>152</v>
+      </c>
+      <c r="N38" s="4">
+        <v>18.852459</v>
       </c>
       <c r="O38" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P38" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q38" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="B39" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="D39" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="E39" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F39" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G39" t="s">
-        <v>164</v>
-      </c>
-      <c r="N39" s="5">
-        <v>18.852459</v>
+        <v>152</v>
+      </c>
+      <c r="N39" s="4">
+        <v>42.622950000000003</v>
       </c>
       <c r="O39" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P39" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q39" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="B40" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="D40" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="E40" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F40" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G40" t="s">
-        <v>164</v>
-      </c>
-      <c r="N40" s="5">
+        <v>152</v>
+      </c>
+      <c r="N40" s="4">
         <v>42.622950000000003</v>
       </c>
       <c r="O40" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P40" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q40" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="B41" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="D41" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="E41" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F41" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G41" t="s">
-        <v>164</v>
-      </c>
-      <c r="N41" s="5">
+        <v>152</v>
+      </c>
+      <c r="N41" s="4">
         <v>42.622950000000003</v>
       </c>
       <c r="O41" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P41" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q41" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="B42" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="D42" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="E42" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F42" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G42" t="s">
-        <v>164</v>
-      </c>
-      <c r="N42" s="5">
+        <v>152</v>
+      </c>
+      <c r="N42" s="4">
         <v>42.622950000000003</v>
       </c>
       <c r="O42" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P42" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q42" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="B43" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="D43" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="E43" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F43" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G43" t="s">
-        <v>164</v>
-      </c>
-      <c r="N43" s="5">
+        <v>152</v>
+      </c>
+      <c r="N43" s="4">
         <v>42.622950000000003</v>
       </c>
       <c r="O43" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P43" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q43" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="B44" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="D44" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="E44" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F44" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G44" t="s">
-        <v>164</v>
-      </c>
-      <c r="N44" s="5">
+        <v>152</v>
+      </c>
+      <c r="N44" s="4">
         <v>42.622950000000003</v>
       </c>
       <c r="O44" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P44" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q44" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="B45" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="D45" t="s">
-        <v>184</v>
+        <v>159</v>
       </c>
       <c r="E45" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F45" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="G45" t="s">
-        <v>164</v>
-      </c>
-      <c r="N45" s="5">
-        <v>42.622950000000003</v>
+        <v>152</v>
+      </c>
+      <c r="H45" t="s">
+        <v>19</v>
+      </c>
+      <c r="I45">
+        <v>25</v>
+      </c>
+      <c r="J45">
+        <v>25</v>
+      </c>
+      <c r="K45">
+        <v>25</v>
+      </c>
+      <c r="N45" s="4">
+        <v>29.508196999999999</v>
       </c>
       <c r="O45" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P45" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q45" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="46" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="B46" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="D46" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="E46" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F46" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="G46" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H46" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I46">
         <v>25</v>
@@ -3222,348 +3160,348 @@
       <c r="K46">
         <v>25</v>
       </c>
-      <c r="N46" s="5">
-        <v>29.508196999999999</v>
+      <c r="N46" s="4">
+        <v>36.065573999999998</v>
       </c>
       <c r="O46" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P46" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q46" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="47" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="B47" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="D47" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E47" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F47" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="G47" t="s">
+        <v>152</v>
+      </c>
+      <c r="H47" t="s">
+        <v>19</v>
+      </c>
+      <c r="I47">
+        <v>10</v>
+      </c>
+      <c r="J47">
+        <v>10</v>
+      </c>
+      <c r="K47">
+        <v>10</v>
+      </c>
+      <c r="N47" s="4">
+        <v>18.852459</v>
+      </c>
+      <c r="O47" t="s">
+        <v>20</v>
+      </c>
+      <c r="P47" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>87</v>
+      </c>
+      <c r="B48" t="s">
+        <v>142</v>
+      </c>
+      <c r="D48" t="s">
+        <v>167</v>
+      </c>
+      <c r="E48" t="s">
+        <v>18</v>
+      </c>
+      <c r="F48" t="s">
+        <v>154</v>
+      </c>
+      <c r="G48" t="s">
+        <v>152</v>
+      </c>
+      <c r="H48" t="s">
+        <v>19</v>
+      </c>
+      <c r="I48">
+        <v>10</v>
+      </c>
+      <c r="J48">
+        <v>10</v>
+      </c>
+      <c r="K48">
+        <v>10</v>
+      </c>
+      <c r="N48" s="4">
+        <v>21.311475000000002</v>
+      </c>
+      <c r="O48" t="s">
+        <v>20</v>
+      </c>
+      <c r="P48" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>88</v>
+      </c>
+      <c r="B49" t="s">
+        <v>143</v>
+      </c>
+      <c r="D49" t="s">
+        <v>158</v>
+      </c>
+      <c r="E49" t="s">
+        <v>18</v>
+      </c>
+      <c r="F49" t="s">
+        <v>154</v>
+      </c>
+      <c r="G49" t="s">
+        <v>152</v>
+      </c>
+      <c r="H49" t="s">
+        <v>19</v>
+      </c>
+      <c r="I49">
+        <v>25</v>
+      </c>
+      <c r="J49">
+        <v>25</v>
+      </c>
+      <c r="K49">
+        <v>25</v>
+      </c>
+      <c r="N49" s="4">
+        <v>39.340000000000003</v>
+      </c>
+      <c r="O49" t="s">
+        <v>20</v>
+      </c>
+      <c r="P49" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>89</v>
+      </c>
+      <c r="B50" t="s">
+        <v>144</v>
+      </c>
+      <c r="D50" t="s">
         <v>164</v>
       </c>
-      <c r="H47" t="s">
-        <v>23</v>
-      </c>
-      <c r="I47">
-        <v>25</v>
-      </c>
-      <c r="J47">
-        <v>25</v>
-      </c>
-      <c r="K47">
-        <v>25</v>
-      </c>
-      <c r="N47" s="5">
-        <v>36.065573999999998</v>
-      </c>
-      <c r="O47" t="s">
-        <v>31</v>
-      </c>
-      <c r="P47" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q47" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="48" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>98</v>
-      </c>
-      <c r="B48" t="s">
-        <v>153</v>
-      </c>
-      <c r="D48" t="s">
-        <v>179</v>
-      </c>
-      <c r="E48" t="s">
-        <v>21</v>
-      </c>
-      <c r="F48" t="s">
-        <v>169</v>
-      </c>
-      <c r="G48" t="s">
-        <v>164</v>
-      </c>
-      <c r="H48" t="s">
-        <v>23</v>
-      </c>
-      <c r="I48">
-        <v>10</v>
-      </c>
-      <c r="J48">
-        <v>10</v>
-      </c>
-      <c r="K48">
-        <v>10</v>
-      </c>
-      <c r="N48" s="5">
-        <v>18.852459</v>
-      </c>
-      <c r="O48" t="s">
-        <v>31</v>
-      </c>
-      <c r="P48" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q48" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="49" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>99</v>
-      </c>
-      <c r="B49" t="s">
+      <c r="E50" t="s">
+        <v>18</v>
+      </c>
+      <c r="F50" t="s">
         <v>154</v>
       </c>
-      <c r="D49" t="s">
-        <v>179</v>
-      </c>
-      <c r="E49" t="s">
-        <v>21</v>
-      </c>
-      <c r="F49" t="s">
-        <v>166</v>
-      </c>
-      <c r="G49" t="s">
-        <v>164</v>
-      </c>
-      <c r="H49" t="s">
-        <v>23</v>
-      </c>
-      <c r="I49">
-        <v>10</v>
-      </c>
-      <c r="J49">
-        <v>10</v>
-      </c>
-      <c r="K49">
-        <v>10</v>
-      </c>
-      <c r="N49" s="5">
-        <v>21.311475000000002</v>
-      </c>
-      <c r="O49" t="s">
-        <v>31</v>
-      </c>
-      <c r="P49" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q49" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="50" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>100</v>
-      </c>
-      <c r="B50" t="s">
-        <v>155</v>
-      </c>
-      <c r="D50" t="s">
+      <c r="G50" t="s">
+        <v>152</v>
+      </c>
+      <c r="H50" t="s">
+        <v>19</v>
+      </c>
+      <c r="I50">
+        <v>10</v>
+      </c>
+      <c r="J50">
+        <v>10</v>
+      </c>
+      <c r="K50">
+        <v>10</v>
+      </c>
+      <c r="N50" s="4">
+        <v>26.23</v>
+      </c>
+      <c r="O50" t="s">
+        <v>20</v>
+      </c>
+      <c r="P50" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>90</v>
+      </c>
+      <c r="B51" t="s">
+        <v>145</v>
+      </c>
+      <c r="D51" t="s">
         <v>170</v>
       </c>
-      <c r="E50" t="s">
-        <v>21</v>
-      </c>
-      <c r="F50" t="s">
-        <v>166</v>
-      </c>
-      <c r="G50" t="s">
-        <v>164</v>
-      </c>
-      <c r="H50" t="s">
-        <v>23</v>
-      </c>
-      <c r="I50">
-        <v>25</v>
-      </c>
-      <c r="J50">
-        <v>25</v>
-      </c>
-      <c r="K50">
-        <v>25</v>
-      </c>
-      <c r="N50" s="5">
-        <v>39.340000000000003</v>
-      </c>
-      <c r="O50" t="s">
-        <v>31</v>
-      </c>
-      <c r="P50" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q50" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="51" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>101</v>
-      </c>
-      <c r="B51" t="s">
-        <v>156</v>
-      </c>
-      <c r="D51" t="s">
-        <v>176</v>
-      </c>
       <c r="E51" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F51" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="G51" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H51" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I51">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J51">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K51">
-        <v>10</v>
-      </c>
-      <c r="N51" s="5">
-        <v>26.23</v>
+        <v>5</v>
+      </c>
+      <c r="N51" s="4">
+        <v>6.5</v>
       </c>
       <c r="O51" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P51" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q51" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B52" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="D52" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="E52" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F52" t="s">
-        <v>169</v>
+        <v>153</v>
       </c>
       <c r="G52" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H52" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I52">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J52">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K52">
-        <v>5</v>
-      </c>
-      <c r="N52" s="5">
-        <v>6.5</v>
+        <v>10</v>
+      </c>
+      <c r="N52" s="4">
+        <v>45</v>
       </c>
       <c r="O52" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P52" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q52" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="53" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="B53" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="D53" t="s">
-        <v>178</v>
+        <v>161</v>
       </c>
       <c r="E53" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F53" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G53" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H53" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I53">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="J53">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="K53">
-        <v>10</v>
-      </c>
-      <c r="N53" s="5">
-        <v>45</v>
+        <v>25</v>
+      </c>
+      <c r="N53" s="4">
+        <v>90</v>
       </c>
       <c r="O53" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P53" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q53" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="B54" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="D54" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="E54" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F54" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G54" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H54" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I54">
         <v>25</v>
@@ -3574,128 +3512,128 @@
       <c r="K54">
         <v>25</v>
       </c>
-      <c r="N54" s="5">
-        <v>90</v>
+      <c r="N54" s="4">
+        <v>137.5</v>
       </c>
       <c r="O54" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P54" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q54" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="55" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="B55" t="s">
+        <v>149</v>
+      </c>
+      <c r="D55" t="s">
+        <v>166</v>
+      </c>
+      <c r="E55" t="s">
+        <v>18</v>
+      </c>
+      <c r="F55" t="s">
+        <v>153</v>
+      </c>
+      <c r="G55" t="s">
+        <v>152</v>
+      </c>
+      <c r="H55" t="s">
+        <v>19</v>
+      </c>
+      <c r="I55">
+        <v>10</v>
+      </c>
+      <c r="J55">
+        <v>10</v>
+      </c>
+      <c r="K55">
+        <v>10</v>
+      </c>
+      <c r="N55" s="4">
+        <v>55</v>
+      </c>
+      <c r="O55" t="s">
+        <v>20</v>
+      </c>
+      <c r="P55" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>95</v>
+      </c>
+      <c r="B56" t="s">
+        <v>150</v>
+      </c>
+      <c r="D56" t="s">
         <v>160</v>
       </c>
-      <c r="D55" t="s">
-        <v>173</v>
-      </c>
-      <c r="E55" t="s">
-        <v>21</v>
-      </c>
-      <c r="F55" t="s">
-        <v>165</v>
-      </c>
-      <c r="G55" t="s">
-        <v>164</v>
-      </c>
-      <c r="H55" t="s">
-        <v>23</v>
-      </c>
-      <c r="I55">
+      <c r="E56" t="s">
+        <v>18</v>
+      </c>
+      <c r="F56" t="s">
+        <v>157</v>
+      </c>
+      <c r="G56" t="s">
+        <v>152</v>
+      </c>
+      <c r="H56" t="s">
+        <v>19</v>
+      </c>
+      <c r="I56">
         <v>25</v>
       </c>
-      <c r="J55">
+      <c r="J56">
         <v>25</v>
       </c>
-      <c r="K55">
+      <c r="K56">
         <v>25</v>
       </c>
-      <c r="N55" s="5">
-        <v>137.5</v>
-      </c>
-      <c r="O55" t="s">
-        <v>31</v>
-      </c>
-      <c r="P55" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q55" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="56" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>106</v>
-      </c>
-      <c r="B56" t="s">
-        <v>161</v>
-      </c>
-      <c r="D56" t="s">
-        <v>178</v>
-      </c>
-      <c r="E56" t="s">
-        <v>21</v>
-      </c>
-      <c r="F56" t="s">
-        <v>165</v>
-      </c>
-      <c r="G56" t="s">
-        <v>164</v>
-      </c>
-      <c r="H56" t="s">
-        <v>23</v>
-      </c>
-      <c r="I56">
-        <v>10</v>
-      </c>
-      <c r="J56">
-        <v>10</v>
-      </c>
-      <c r="K56">
-        <v>10</v>
-      </c>
-      <c r="N56" s="5">
-        <v>55</v>
+      <c r="N56" s="4">
+        <v>12</v>
       </c>
       <c r="O56" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P56" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q56" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="57" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="B57" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="D57" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="E57" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F57" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="G57" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H57" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I57">
         <v>25</v>
@@ -3706,69 +3644,20 @@
       <c r="K57">
         <v>25</v>
       </c>
-      <c r="N57" s="5">
-        <v>12</v>
+      <c r="N57" s="4">
+        <v>28.69</v>
       </c>
       <c r="O57" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="P57" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="Q57" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="58" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>108</v>
-      </c>
-      <c r="B58" t="s">
-        <v>163</v>
-      </c>
-      <c r="D58" t="s">
-        <v>171</v>
-      </c>
-      <c r="E58" t="s">
-        <v>21</v>
-      </c>
-      <c r="F58" t="s">
-        <v>167</v>
-      </c>
-      <c r="G58" t="s">
-        <v>164</v>
-      </c>
-      <c r="H58" t="s">
-        <v>23</v>
-      </c>
-      <c r="I58">
-        <v>25</v>
-      </c>
-      <c r="J58">
-        <v>25</v>
-      </c>
-      <c r="K58">
-        <v>25</v>
-      </c>
-      <c r="N58" s="5">
-        <v>28.69</v>
-      </c>
-      <c r="O58" t="s">
-        <v>31</v>
-      </c>
-      <c r="P58" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q58" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R58" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="3">
-      <filters blank="1"/>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
   <legacyDrawing r:id="rId1"/>
@@ -3785,27 +3674,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>34</v>
+      <c r="A1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -3813,7 +3702,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -3821,7 +3710,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -3829,7 +3718,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -3837,7 +3726,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -3845,7 +3734,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -3853,7 +3742,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -3861,7 +3750,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -3869,7 +3758,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -3877,7 +3766,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -3885,7 +3774,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -3893,7 +3782,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -3901,7 +3790,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -3909,7 +3798,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -3917,7 +3806,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -3925,7 +3814,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -3933,7 +3822,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>